<commit_message>
Updated RFCC CarePlan Model File with 6 tabs
</commit_message>
<xml_diff>
--- a/ontology/care-plan/RFCC_CarePlan_Model.xlsx.xlsx
+++ b/ontology/care-plan/RFCC_CarePlan_Model.xlsx.xlsx
@@ -1,13 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repositories_GitHub\ucm\ontology\care-plan\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{853C452C-A869-4679-A611-0EFDE0A99F2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="3570" yWindow="720" windowWidth="23130" windowHeight="13425" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="01_Definition" sheetId="1" r:id="rId1"/>
+    <sheet name="02_Participants" sheetId="2" r:id="rId2"/>
+    <sheet name="03_Shared_Characteristics" sheetId="3" r:id="rId3"/>
+    <sheet name="04_Elements" sheetId="4" r:id="rId4"/>
+    <sheet name="05_Participant_to_Element" sheetId="5" r:id="rId5"/>
+    <sheet name="06_Terminology_Bindings" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -18,12 +29,298 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="89">
+  <si>
+    <t>Purpose: Who can creae/update/view elements</t>
+  </si>
+  <si>
+    <t>Participant</t>
+  </si>
+  <si>
+    <t>Element</t>
+  </si>
+  <si>
+    <t>Create</t>
+  </si>
+  <si>
+    <t>Update</t>
+  </si>
+  <si>
+    <t>View</t>
+  </si>
+  <si>
+    <t>Monitor</t>
+  </si>
+  <si>
+    <t>Purpose:</t>
+  </si>
+  <si>
+    <t>RFCC_ID</t>
+  </si>
+  <si>
+    <t>Concept</t>
+  </si>
+  <si>
+    <t>Code_System</t>
+  </si>
+  <si>
+    <t>Code</t>
+  </si>
+  <si>
+    <t>Display</t>
+  </si>
+  <si>
+    <t>FHIR Resource</t>
+  </si>
+  <si>
+    <t>Bindin Type</t>
+  </si>
+  <si>
+    <t>Verification Status</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Purpose: What a care plan contains.</t>
+  </si>
+  <si>
+    <t>Element_ID</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Problems</t>
+  </si>
+  <si>
+    <t>Goals</t>
+  </si>
+  <si>
+    <t>Objectives</t>
+  </si>
+  <si>
+    <t>Interventions</t>
+  </si>
+  <si>
+    <t>Actions</t>
+  </si>
+  <si>
+    <t>Services</t>
+  </si>
+  <si>
+    <t>Tasks</t>
+  </si>
+  <si>
+    <t>Responsibilities</t>
+  </si>
+  <si>
+    <t>Referrals</t>
+  </si>
+  <si>
+    <t>Outcomes</t>
+  </si>
+  <si>
+    <t>Follow-up</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Needs</t>
+  </si>
+  <si>
+    <t>ELM-001</t>
+  </si>
+  <si>
+    <t>ELM-002</t>
+  </si>
+  <si>
+    <t>ELM-003</t>
+  </si>
+  <si>
+    <t>ELM-004</t>
+  </si>
+  <si>
+    <t>ELM-005</t>
+  </si>
+  <si>
+    <t>ELM-006</t>
+  </si>
+  <si>
+    <t>ELM-007</t>
+  </si>
+  <si>
+    <t>ELM-008</t>
+  </si>
+  <si>
+    <t>ELM-009</t>
+  </si>
+  <si>
+    <t>ELM-010</t>
+  </si>
+  <si>
+    <t>ELM-011</t>
+  </si>
+  <si>
+    <t>ELM-012</t>
+  </si>
+  <si>
+    <t>ELM-013</t>
+  </si>
+  <si>
+    <t>Purpose: What all care plans have.</t>
+  </si>
+  <si>
+    <t>Characteristic ID</t>
+  </si>
+  <si>
+    <t>Characteristic</t>
+  </si>
+  <si>
+    <t>CHAR-001</t>
+  </si>
+  <si>
+    <t>CHAR-002</t>
+  </si>
+  <si>
+    <t>Person-Centered</t>
+  </si>
+  <si>
+    <t>Longitudinal</t>
+  </si>
+  <si>
+    <t>Shared</t>
+  </si>
+  <si>
+    <t>Goal-Oriented</t>
+  </si>
+  <si>
+    <t>Dynamic</t>
+  </si>
+  <si>
+    <t>Multi-Participant</t>
+  </si>
+  <si>
+    <t>Actionable</t>
+  </si>
+  <si>
+    <t>Coordinated</t>
+  </si>
+  <si>
+    <t>Trackable</t>
+  </si>
+  <si>
+    <t>CHAR-003</t>
+  </si>
+  <si>
+    <t>CHAR-004</t>
+  </si>
+  <si>
+    <t>CHAR-005</t>
+  </si>
+  <si>
+    <t>CHAR-006</t>
+  </si>
+  <si>
+    <t>CHAR-007</t>
+  </si>
+  <si>
+    <t>CHAR-008</t>
+  </si>
+  <si>
+    <t>CHAR-009</t>
+  </si>
+  <si>
+    <t>Purpose: Who interacts with care plans.</t>
+  </si>
+  <si>
+    <t>Participant ID</t>
+  </si>
+  <si>
+    <t>Definition</t>
+  </si>
+  <si>
+    <t>Reference</t>
+  </si>
+  <si>
+    <t>PAR-001</t>
+  </si>
+  <si>
+    <t>PAR-002</t>
+  </si>
+  <si>
+    <t>Individual</t>
+  </si>
+  <si>
+    <t>Caregiver</t>
+  </si>
+  <si>
+    <t>Care Coordinaiton an Support Personnel</t>
+  </si>
+  <si>
+    <t>Clinician</t>
+  </si>
+  <si>
+    <t>Community Organization</t>
+  </si>
+  <si>
+    <t>Service Provider</t>
+  </si>
+  <si>
+    <t>PAR-003</t>
+  </si>
+  <si>
+    <t>PAR-004</t>
+  </si>
+  <si>
+    <t>PAR-005</t>
+  </si>
+  <si>
+    <t>PAR-006</t>
+  </si>
+  <si>
+    <t>Purpose: Define what Care Plan means</t>
+  </si>
+  <si>
+    <t>Scope</t>
+  </si>
+  <si>
+    <t>Shared Care Plan</t>
+  </si>
+  <si>
+    <t>A structured and evolving plan that records goals, neds, problems, interventions, responsibilities, services, and outcomes contributed to and used by multiple participants to support coordinated and person-centered care across settings and organizations.</t>
+  </si>
+  <si>
+    <t>RFCC / UCM</t>
+  </si>
+  <si>
+    <t>TBD</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -49,8 +346,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -330,10 +637,464 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="18.140625" customWidth="1"/>
+    <col min="2" max="2" width="72.42578125" customWidth="1"/>
+    <col min="3" max="3" width="15.5703125" customWidth="1"/>
+    <col min="4" max="4" width="21.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" s="1" customFormat="1" ht="81" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>88</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{052D1280-BFD6-45F2-A5EB-7BCFD167F59C}">
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="14.7109375" customWidth="1"/>
+    <col min="2" max="2" width="39.42578125" customWidth="1"/>
+    <col min="3" max="3" width="21.28515625" customWidth="1"/>
+    <col min="4" max="4" width="19.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>71</v>
+      </c>
+      <c r="B3" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B4" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>79</v>
+      </c>
+      <c r="B5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>80</v>
+      </c>
+      <c r="B6" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>81</v>
+      </c>
+      <c r="B7" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>82</v>
+      </c>
+      <c r="B8" t="s">
+        <v>78</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E0B982B-7339-4140-A4E9-1991992E23F5}">
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="17" customWidth="1"/>
+    <col min="2" max="2" width="17.85546875" customWidth="1"/>
+    <col min="3" max="3" width="42.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>60</v>
+      </c>
+      <c r="B5" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>61</v>
+      </c>
+      <c r="B6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>62</v>
+      </c>
+      <c r="B7" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>63</v>
+      </c>
+      <c r="B8" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>64</v>
+      </c>
+      <c r="B9" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>65</v>
+      </c>
+      <c r="B10" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>66</v>
+      </c>
+      <c r="B11" t="s">
+        <v>59</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B9E8638-5AFE-4FE4-AE18-3350BD5FBC6F}">
+  <dimension ref="A1:C15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="14.42578125" customWidth="1"/>
+    <col min="2" max="2" width="21.28515625" customWidth="1"/>
+    <col min="3" max="3" width="35.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>37</v>
+      </c>
+      <c r="B7" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B8" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>39</v>
+      </c>
+      <c r="B9" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>40</v>
+      </c>
+      <c r="B10" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>41</v>
+      </c>
+      <c r="B11" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>42</v>
+      </c>
+      <c r="B12" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B13" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>44</v>
+      </c>
+      <c r="B14" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>45</v>
+      </c>
+      <c r="B15" t="s">
+        <v>32</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50E747BE-7B2A-481F-A83F-99E6BA47E654}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15.85546875" customWidth="1"/>
+    <col min="2" max="2" width="15.7109375" customWidth="1"/>
+    <col min="3" max="3" width="18.5703125" customWidth="1"/>
+    <col min="4" max="4" width="15.7109375" customWidth="1"/>
+    <col min="5" max="5" width="13.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F507E89-610B-4D2D-A0EB-9D9EE3928082}">
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr defaultColWidth="14" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="6" max="6" width="18.7109375" customWidth="1"/>
+    <col min="8" max="8" width="19.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Care Plan Excel Tabs updated
</commit_message>
<xml_diff>
--- a/ontology/care-plan/RFCC_CarePlan_Model.xlsx.xlsx
+++ b/ontology/care-plan/RFCC_CarePlan_Model.xlsx.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repositories_GitHub\ucm\ontology\care-plan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{853C452C-A869-4679-A611-0EFDE0A99F2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C1593B0-FE40-4141-88D1-104895D55BDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3570" yWindow="720" windowWidth="23130" windowHeight="13425" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3570" yWindow="720" windowWidth="23130" windowHeight="13425" firstSheet="4" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="01_Definition" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,8 @@
     <sheet name="04_Elements" sheetId="4" r:id="rId4"/>
     <sheet name="05_Participant_to_Element" sheetId="5" r:id="rId5"/>
     <sheet name="06_Terminology_Bindings" sheetId="6" r:id="rId6"/>
+    <sheet name="07_Modality" sheetId="7" r:id="rId7"/>
+    <sheet name="08_Element_to_Modality" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -30,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="151">
   <si>
     <t>Purpose: Who can creae/update/view elements</t>
   </si>
@@ -297,6 +299,192 @@
   </si>
   <si>
     <t>TBD</t>
+  </si>
+  <si>
+    <t>Organized around individual goals, preferences, values, needs, and outcomes.</t>
+  </si>
+  <si>
+    <t>ACL</t>
+  </si>
+  <si>
+    <t>Maintained and updated over time across episodes and settings.</t>
+  </si>
+  <si>
+    <t>CMS</t>
+  </si>
+  <si>
+    <t>Intended to support contributions, use, and coordination across participants and organizations</t>
+  </si>
+  <si>
+    <t>HL7</t>
+  </si>
+  <si>
+    <t>Structured to achieve defined outcomes and objectives.</t>
+  </si>
+  <si>
+    <t>Supports updates as conditions, needs, or services change.</t>
+  </si>
+  <si>
+    <t>AHRQ</t>
+  </si>
+  <si>
+    <t>Multiple participants may contribute to and use the plan.</t>
+  </si>
+  <si>
+    <t>Supports execution and coordination of activities and services.</t>
+  </si>
+  <si>
+    <t>FHIR</t>
+  </si>
+  <si>
+    <t>Supports alignment across participatns and services.</t>
+  </si>
+  <si>
+    <t>Supports monitoring status. Progress, and outcomes.</t>
+  </si>
+  <si>
+    <t>Interoperable</t>
+  </si>
+  <si>
+    <t>Supports exchange across systems and organizations.</t>
+  </si>
+  <si>
+    <t>CHAR-010</t>
+  </si>
+  <si>
+    <t>Modality_ID</t>
+  </si>
+  <si>
+    <t>Modality</t>
+  </si>
+  <si>
+    <t>Example</t>
+  </si>
+  <si>
+    <t>MOD-001</t>
+  </si>
+  <si>
+    <t>In-Person</t>
+  </si>
+  <si>
+    <t>Care Planning occurs through physical interaction.</t>
+  </si>
+  <si>
+    <t>Office Visit</t>
+  </si>
+  <si>
+    <t>Virtual</t>
+  </si>
+  <si>
+    <t>Care planning occures through telehealth or remote engagement</t>
+  </si>
+  <si>
+    <t>Video conference</t>
+  </si>
+  <si>
+    <t>Hybrid</t>
+  </si>
+  <si>
+    <t>Combination of in-person and virtual participation</t>
+  </si>
+  <si>
+    <t>Care team + telehealth</t>
+  </si>
+  <si>
+    <t>Synchronous</t>
+  </si>
+  <si>
+    <t>Participants contribute over time independently</t>
+  </si>
+  <si>
+    <t>Shared updates</t>
+  </si>
+  <si>
+    <t>Asynchronous</t>
+  </si>
+  <si>
+    <t>Participants contribute at the same time.</t>
+  </si>
+  <si>
+    <t>Team meeting</t>
+  </si>
+  <si>
+    <t>Document-Based</t>
+  </si>
+  <si>
+    <t>Plan maintained through exchanged documents.</t>
+  </si>
+  <si>
+    <t>Care summary</t>
+  </si>
+  <si>
+    <t>System-based</t>
+  </si>
+  <si>
+    <t>Plan maintained through shared systems/platforms.</t>
+  </si>
+  <si>
+    <t>Shared HER</t>
+  </si>
+  <si>
+    <t>Participant-Managed</t>
+  </si>
+  <si>
+    <t>Individual manages updates and participation.</t>
+  </si>
+  <si>
+    <t>Patient-entered plan</t>
+  </si>
+  <si>
+    <t>Coordinaed</t>
+  </si>
+  <si>
+    <t>Updates managed across participants and organizations</t>
+  </si>
+  <si>
+    <t>Care Coordination workflow</t>
+  </si>
+  <si>
+    <t>MOD-002</t>
+  </si>
+  <si>
+    <t>MOD-003</t>
+  </si>
+  <si>
+    <t>MOD-004</t>
+  </si>
+  <si>
+    <t>MOD-005</t>
+  </si>
+  <si>
+    <t>MOD-006</t>
+  </si>
+  <si>
+    <t>MOD-007</t>
+  </si>
+  <si>
+    <t>MOD-008</t>
+  </si>
+  <si>
+    <t>MOD-009</t>
+  </si>
+  <si>
+    <t>Supported Modality</t>
+  </si>
+  <si>
+    <t>Required</t>
+  </si>
+  <si>
+    <t>All</t>
+  </si>
+  <si>
+    <t>Follow Up</t>
+  </si>
+  <si>
+    <t>System-Based</t>
+  </si>
+  <si>
+    <t>Purpose: Attribute of the care plan to represent how is the care plan delivered / coordinated / represented (operatates)?</t>
   </si>
 </sst>
 </file>
@@ -326,12 +514,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -346,7 +540,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -358,6 +552,19 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -771,102 +978,184 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E0B982B-7339-4140-A4E9-1991992E23F5}">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17" customWidth="1"/>
-    <col min="2" max="2" width="17.85546875" customWidth="1"/>
-    <col min="3" max="3" width="42.5703125" customWidth="1"/>
+    <col min="1" max="1" width="17" style="1" customWidth="1"/>
+    <col min="2" max="2" width="17.85546875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="55.140625" style="3" customWidth="1"/>
+    <col min="4" max="4" width="16.7109375" style="5" customWidth="1"/>
+    <col min="5" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="7" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="D2" s="8" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="1" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="C3" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="1" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="C4" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="1" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="C5" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="1" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="C6" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="1" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="C7" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="1" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+      <c r="C8" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="C9" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="1" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="C10" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="1" t="s">
         <v>59</v>
       </c>
-    </row>
+      <c r="C11" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="33" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="14" spans="1:4" ht="33" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="1:4" ht="33" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="16" spans="1:4" ht="33" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="17" ht="33" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="18" ht="33" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="19" ht="33" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="20" ht="33" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="21" ht="33" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1097,4 +1386,235 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{035054EA-E6E1-4FE2-B735-7F5F2603B7E4}">
+  <dimension ref="A1:D20"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.5703125" customWidth="1"/>
+    <col min="2" max="2" width="23.7109375" customWidth="1"/>
+    <col min="3" max="3" width="60" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" s="1" customFormat="1" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>109</v>
+      </c>
+      <c r="B3" t="s">
+        <v>110</v>
+      </c>
+      <c r="C3" t="s">
+        <v>111</v>
+      </c>
+      <c r="D3" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>137</v>
+      </c>
+      <c r="B4" t="s">
+        <v>113</v>
+      </c>
+      <c r="C4" t="s">
+        <v>114</v>
+      </c>
+      <c r="D4" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>138</v>
+      </c>
+      <c r="B5" t="s">
+        <v>116</v>
+      </c>
+      <c r="C5" t="s">
+        <v>117</v>
+      </c>
+      <c r="D5" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>139</v>
+      </c>
+      <c r="B6" t="s">
+        <v>119</v>
+      </c>
+      <c r="C6" t="s">
+        <v>123</v>
+      </c>
+      <c r="D6" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>140</v>
+      </c>
+      <c r="B7" t="s">
+        <v>122</v>
+      </c>
+      <c r="C7" t="s">
+        <v>120</v>
+      </c>
+      <c r="D7" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>141</v>
+      </c>
+      <c r="B8" t="s">
+        <v>125</v>
+      </c>
+      <c r="C8" t="s">
+        <v>126</v>
+      </c>
+      <c r="D8" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>142</v>
+      </c>
+      <c r="B9" t="s">
+        <v>128</v>
+      </c>
+      <c r="C9" t="s">
+        <v>129</v>
+      </c>
+      <c r="D9" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>143</v>
+      </c>
+      <c r="B10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C10" t="s">
+        <v>132</v>
+      </c>
+      <c r="D10" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>144</v>
+      </c>
+      <c r="B11" t="s">
+        <v>134</v>
+      </c>
+      <c r="C11" t="s">
+        <v>135</v>
+      </c>
+      <c r="D11" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="13" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="14" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="16" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="18" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="19" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CEB7FA1-CB43-4C0E-9BCD-F484DAFDBEBA}">
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr defaultColWidth="12.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="33.7109375" customWidth="1"/>
+    <col min="3" max="3" width="19.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>146</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>148</v>
+      </c>
+      <c r="B3" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" t="s">
+        <v>149</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>